<commit_message>
Bold Others: in Q11; hide module section headers when module not selected; republish xlsx
</commit_message>
<xml_diff>
--- a/cat0200_import.xlsx
+++ b/cat0200_import.xlsx
@@ -1236,7 +1236,11 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr"/>
-      <c r="B17" s="2" t="inlineStr"/>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>CAT0200-13-finance</t>
+        </is>
+      </c>
       <c r="C17" s="2" t="inlineStr"/>
       <c r="D17" s="2" t="inlineStr">
         <is>
@@ -1356,7 +1360,11 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr"/>
-      <c r="B20" s="2" t="inlineStr"/>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>CAT0200-13-sales_crm</t>
+        </is>
+      </c>
       <c r="C20" s="2" t="inlineStr"/>
       <c r="D20" s="2" t="inlineStr">
         <is>
@@ -1524,7 +1532,11 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr"/>
-      <c r="B24" s="2" t="inlineStr"/>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>CAT0200-13-supply_chain</t>
+        </is>
+      </c>
       <c r="C24" s="2" t="inlineStr"/>
       <c r="D24" s="2" t="inlineStr">
         <is>
@@ -1740,7 +1752,11 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr"/>
-      <c r="B29" s="2" t="inlineStr"/>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>CAT0200-13-hr</t>
+        </is>
+      </c>
       <c r="C29" s="2" t="inlineStr"/>
       <c r="D29" s="2" t="inlineStr">
         <is>
@@ -2192,7 +2208,11 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr"/>
-      <c r="B39" s="2" t="inlineStr"/>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>CAT0200-13-manufacturing</t>
+        </is>
+      </c>
       <c r="C39" s="2" t="inlineStr"/>
       <c r="D39" s="2" t="inlineStr">
         <is>
@@ -2496,7 +2516,11 @@
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr"/>
-      <c r="B46" s="2" t="inlineStr"/>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>CAT0200-13-fleet</t>
+        </is>
+      </c>
       <c r="C46" s="2" t="inlineStr"/>
       <c r="D46" s="2" t="inlineStr">
         <is>
@@ -2612,7 +2636,11 @@
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr"/>
-      <c r="B49" s="2" t="inlineStr"/>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>CAT0200-13-field_service</t>
+        </is>
+      </c>
       <c r="C49" s="2" t="inlineStr"/>
       <c r="D49" s="2" t="inlineStr">
         <is>
@@ -2684,7 +2712,11 @@
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr"/>
-      <c r="B51" s="2" t="inlineStr"/>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>CAT0200-13-project</t>
+        </is>
+      </c>
       <c r="C51" s="2" t="inlineStr"/>
       <c r="D51" s="2" t="inlineStr">
         <is>
@@ -2756,7 +2788,11 @@
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr"/>
-      <c r="B53" s="2" t="inlineStr"/>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>CAT0200-13-asset</t>
+        </is>
+      </c>
       <c r="C53" s="2" t="inlineStr"/>
       <c r="D53" s="2" t="inlineStr">
         <is>
@@ -2828,7 +2864,11 @@
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr"/>
-      <c r="B55" s="2" t="inlineStr"/>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>CAT0200-13.1-Yes</t>
+        </is>
+      </c>
       <c r="C55" s="2" t="inlineStr"/>
       <c r="D55" s="2" t="inlineStr">
         <is>
@@ -5249,7 +5289,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Others: Please Specify</t>
+          <t>__Others:__ Please Specify</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">

</xml_diff>

<commit_message>
UK spelling + remove em-dashes/AI filler from CAT0200 content; republish xlsx
</commit_message>
<xml_diff>
--- a/cat0200_import.xlsx
+++ b/cat0200_import.xlsx
@@ -605,7 +605,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Can your solution demonstrate compliance with the following Personal Data Protection requirements?&lt;br/&gt;&lt;br/&gt;Digital solutions that collect, use, disclose, process or dispose personal data should incorporate features that support the obligations under the Personal Data Protection Act (2020).&lt;br/&gt;&lt;br/&gt;To comply with this requirement, you MUST complete the Personal Data Protection Requirements form at https://go.gov.sg/pdp.&lt;br/&gt;&lt;br/&gt;Please note that this requirement is **Mandatory** for the following iERP modules:&lt;br/&gt;**(1) Sales &amp; CRM Module**&lt;br/&gt;**(2) HR Management**</t>
+          <t>Can your solution demonstrate compliance with the following Personal Data Protection requirements?&lt;br/&gt;&lt;br/&gt;Digital solutions that collect, use, disclose, process or dispose personal data should incorporate features that support the obligations under the Personal Data Protection Act (2020).&lt;br/&gt;&lt;br/&gt;To comply with this requirement, you MUST complete the Personal Data Protection Requirements form at https://go.gov.sg/pdp.&lt;br/&gt;&lt;br/&gt;**Note:** this requirement is **Mandatory** for the following iERP modules:&lt;br/&gt;**(1) Sales &amp; CRM Module**&lt;br/&gt;**(2) HR Management**</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -2489,7 +2489,7 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Does your module centralize routing and work instructions—including engineering drawing, tool, and manpower management—while governing revisions through engineering change management, and also have other relevant features that facilitate &amp; streamline product lifecycle management (PLM) workflows?</t>
+          <t>Does your module centralise routing and work instructions (including engineering drawing, tool, and manpower management) while governing revisions through engineering change management, and also have other relevant features that facilitate &amp; streamline product lifecycle management (PLM) workflows?</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -2565,7 +2565,7 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Does your module utilize telematics and GPS for real-time fleet tracking, automate dispatch and dynamic route planning using live traffic data, and also have other relevant features that facilitate &amp; streamline fleet management and transport operations?</t>
+          <t>Does your module use telematics and GPS for real-time fleet tracking, automate dispatch and dynamic route planning using live traffic data, and also have other relevant features that facilitate &amp; streamline fleet management and transport operations?</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -2837,7 +2837,7 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Does your module track the centralized lifecycle of assets from procurement to decommissioning, automate maintenance scheduling based on usage thresholds, and continuously monitor equipment utilization and compliance histories across multiple sites, and also have other relevant features that facilitate &amp; streamline asset management?</t>
+          <t>Does your module track the centralised lifecycle of assets from procurement to decommissioning, automate maintenance scheduling based on usage thresholds, and continuously monitor equipment utilisation and compliance histories across multiple sites, and also have other relevant features that facilitate &amp; streamline asset management?</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -3397,7 +3397,7 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Which third-party ERP module/application types can your solution integrate with?&lt;br/&gt;&lt;br/&gt;Please select a minimum of at least 1 module.&lt;br/&gt;&lt;br/&gt;**Note 1:** You can only be qualified for up to the 9 modules defined above — submissions for other undefined modules not in the list will not be accepted.</t>
+          <t>Which third-party ERP module/application types can your solution integrate with?&lt;br/&gt;&lt;br/&gt;Please select a minimum of at least 1 module.&lt;br/&gt;&lt;br/&gt;**Note 1:** You can only be qualified for up to the 9 modules defined above. Submissions for other undefined modules not in the list will not be accepted.</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">

</xml_diff>

<commit_message>
AI-Others optional upload (Q12); relocate Others-module opt-in (Q13.1); republish xlsx
</commit_message>
<xml_diff>
--- a/cat0200_import.xlsx
+++ b/cat0200_import.xlsx
@@ -1142,8 +1142,16 @@
       </c>
       <c r="J14" s="2" t="inlineStr"/>
       <c r="K14" s="2" t="inlineStr"/>
-      <c r="L14" s="2" t="inlineStr"/>
-      <c r="M14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>Attach supporting document</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -1169,7 +1177,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Which ERP modules does your solution provide?&lt;br/&gt;&lt;br/&gt;Please select a minimum of at least 3 modules.&lt;br/&gt;&lt;br/&gt;**Note:** To submit an additional module not covered in the list above, use the "Others Module" question that follows. "Others" does not count toward the minimum of 3 modules.</t>
+          <t>Which ERP modules does your solution provide?&lt;br/&gt;&lt;br/&gt;Please select a minimum of at least 3 modules.&lt;br/&gt;&lt;br/&gt;**Note:** To submit an additional module not covered in the list above, use the "Others Module" question shown after the module sections. "Others" does not count toward the minimum of 3 modules.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -1195,30 +1203,22 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>CAT0200-13.1</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr"/>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Preferred</t>
-        </is>
-      </c>
+      <c r="A16" s="2" t="inlineStr"/>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>CAT0200-13-finance</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr"/>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Others Module</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>Do you also provide an ERP module that is not covered by the list above (an "Others" module)?&lt;br/&gt;&lt;br/&gt;You may submit at most 1 "Others" module, and it does not count toward the minimum of 3 modules above. Select "Yes" to declare it below.</t>
-        </is>
-      </c>
+          <t>Financial Management Module</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Radio</t>
+          <t>Label</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr"/>
@@ -1228,44 +1228,60 @@
       <c r="K16" s="2" t="inlineStr"/>
       <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="2" t="inlineStr"/>
-      <c r="N16" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="N16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr"/>
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>CAT0200-14</t>
+        </is>
+      </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
           <t>CAT0200-13-finance</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr"/>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Financial Management Module</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr"/>
+          <t>Core Finance Module Features</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Does your module integrate a general ledger, customer invoicing, vendor bills, bank-ledger matching and also have other relevant features that facilitate &amp; streamline core accounting processes?</t>
+        </is>
+      </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Label</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr"/>
+          <t>Checkbox</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="H17" s="2" t="inlineStr"/>
       <c r="I17" s="2" t="inlineStr"/>
       <c r="J17" s="2" t="inlineStr"/>
       <c r="K17" s="2" t="inlineStr"/>
       <c r="L17" s="2" t="inlineStr"/>
       <c r="M17" s="2" t="inlineStr"/>
-      <c r="N17" s="2" t="inlineStr"/>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-14</t>
+          <t>CAT0200-15</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1280,12 +1296,12 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Core Finance Module Features</t>
+          <t>InvoiceNow-Ready Solution Provider Accreditation</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Does your module integrate a general ledger, customer invoicing, vendor bills, bank-ledger matching and also have other relevant features that facilitate &amp; streamline core accounting processes?</t>
+          <t>Is your solution listed on IMDA InvoiceNow-Ready Solution Provider (IRSP) Listing?&lt;br/&gt;&lt;br/&gt;[1] If you are the Product Principal of the solution, you are required to be accredited as an IRSP by IMDA. [2] If you are the reseller of the solution, your Solution Product Principal must declare to IMDA that you are an authorised reseller of their solution.&lt;br/&gt;&lt;br/&gt;**Note:** For more information on InvoiceNow, refer to: Becoming an InvoiceNow-Ready Solution Provider | E-invoicing | IMDA (https://www.imda.gov.sg/how-we-can-help/nationwide-e-invoicing-framework/becoming-an-invoicenow-ready-solution-provider)</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1311,90 +1327,90 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>CAT0200-15</t>
-        </is>
-      </c>
+      <c r="A19" s="2" t="inlineStr"/>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-13-finance</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Mandatory</t>
-        </is>
-      </c>
+          <t>CAT0200-13-sales_crm</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr"/>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>InvoiceNow-Ready Solution Provider Accreditation</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>Is your solution listed on IMDA InvoiceNow-Ready Solution Provider (IRSP) Listing?&lt;br/&gt;&lt;br/&gt;[1] If you are the Product Principal of the solution, you are required to be accredited as an IRSP by IMDA. [2] If you are the reseller of the solution, your Solution Product Principal must declare to IMDA that you are an authorised reseller of their solution.&lt;br/&gt;&lt;br/&gt;**Note:** For more information on InvoiceNow, refer to: Becoming an InvoiceNow-Ready Solution Provider | E-invoicing | IMDA (https://www.imda.gov.sg/how-we-can-help/nationwide-e-invoicing-framework/becoming-an-invoicenow-ready-solution-provider)</t>
-        </is>
-      </c>
+          <t>Sales &amp; CRM Module</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Checkbox</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr"/>
       <c r="H19" s="2" t="inlineStr"/>
       <c r="I19" s="2" t="inlineStr"/>
       <c r="J19" s="2" t="inlineStr"/>
       <c r="K19" s="2" t="inlineStr"/>
       <c r="L19" s="2" t="inlineStr"/>
       <c r="M19" s="2" t="inlineStr"/>
-      <c r="N19" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="N19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr"/>
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>CAT0200-16</t>
+        </is>
+      </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
           <t>CAT0200-13-sales_crm</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr"/>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Sales &amp; CRM Module</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr"/>
+          <t>Sales &amp; CRM - Sub-Modules</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Which of these sub-modules within the Sales &amp; CRM module do you provide?&lt;br/&gt;&lt;br/&gt;**Note:** You have to select at least 1 option to qualify for this module.</t>
+        </is>
+      </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Label</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr"/>
+          <t>Checkbox</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="H20" s="2" t="inlineStr"/>
       <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="inlineStr"/>
       <c r="K20" s="2" t="inlineStr"/>
       <c r="L20" s="2" t="inlineStr"/>
       <c r="M20" s="2" t="inlineStr"/>
-      <c r="N20" s="2" t="inlineStr"/>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-16</t>
+          <t>CAT0200-17</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-13-sales_crm</t>
+          <t>CAT0200-16-sales</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -1404,12 +1420,12 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Sales &amp; CRM - Sub-Modules</t>
+          <t>Sales Features - Elaboration</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Which of these sub-modules within the Sales &amp; CRM module do you provide?&lt;br/&gt;&lt;br/&gt;**Note:** You have to select at least 1 option to qualify for this module.</t>
+          <t>Does your module record customer orders, generate invoices and link payment statuses and also have other relevant features that facilitate &amp; streamline the order-to-cash workflow?</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -1437,12 +1453,12 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-17</t>
+          <t>CAT0200-18</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-16-sales</t>
+          <t>CAT0200-16-crm</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -1452,12 +1468,12 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Sales Features - Elaboration</t>
+          <t>Customer Relationship Management (CRM) - Elaboration Features</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Does your module record customer orders, generate invoices and link payment statuses and also have other relevant features that facilitate &amp; streamline the order-to-cash workflow?</t>
+          <t>Does your module maintain customer records &amp; interactions, as well as effectively capture leads and converting them into active opportunities, and also have other relevant features that facilitate &amp; streamline customer and lead management?</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -1483,90 +1499,90 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>CAT0200-18</t>
-        </is>
-      </c>
+      <c r="A23" s="2" t="inlineStr"/>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-16-crm</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>Mandatory</t>
-        </is>
-      </c>
+          <t>CAT0200-13-supply_chain</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr"/>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Customer Relationship Management (CRM) - Elaboration Features</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>Does your module maintain customer records &amp; interactions, as well as effectively capture leads and converting them into active opportunities, and also have other relevant features that facilitate &amp; streamline customer and lead management?</t>
-        </is>
-      </c>
+          <t>Supply Chain &amp; Inventory Management Module</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Checkbox</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr"/>
       <c r="H23" s="2" t="inlineStr"/>
       <c r="I23" s="2" t="inlineStr"/>
       <c r="J23" s="2" t="inlineStr"/>
       <c r="K23" s="2" t="inlineStr"/>
       <c r="L23" s="2" t="inlineStr"/>
       <c r="M23" s="2" t="inlineStr"/>
-      <c r="N23" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="N23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr"/>
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>CAT0200-19</t>
+        </is>
+      </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
           <t>CAT0200-13-supply_chain</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr"/>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Supply Chain &amp; Inventory Management Module</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr"/>
+          <t>Supply Chain &amp; Inventory Management - Sub-Modules</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Which of these sub-modules within the Supply Chain &amp; Inventory Management module do you provide?&lt;br/&gt;&lt;br/&gt;**Note:** You have to select at least 1 option to qualify for this module.</t>
+        </is>
+      </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Label</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr"/>
+          <t>Checkbox</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="H24" s="2" t="inlineStr"/>
       <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="2" t="inlineStr"/>
       <c r="K24" s="2" t="inlineStr"/>
       <c r="L24" s="2" t="inlineStr"/>
       <c r="M24" s="2" t="inlineStr"/>
-      <c r="N24" s="2" t="inlineStr"/>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-19</t>
+          <t>CAT0200-20</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-13-supply_chain</t>
+          <t>CAT0200-19-procurement</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -1576,12 +1592,12 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Supply Chain &amp; Inventory Management - Sub-Modules</t>
+          <t>Procurement &amp; Purchasing Features - Elaboration</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Which of these sub-modules within the Supply Chain &amp; Inventory Management module do you provide?&lt;br/&gt;&lt;br/&gt;**Note:** You have to select at least 1 option to qualify for this module.</t>
+          <t>Does your module seamlessly track purchase orders from initial creation all the way through to final invoice payment, as well as maintain comprehensive vendor master records, and also have other relevant features that streamline supplier management?</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -1609,12 +1625,12 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-20</t>
+          <t>CAT0200-21</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-19-procurement</t>
+          <t>CAT0200-19-warehouse</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1624,12 +1640,12 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Procurement &amp; Purchasing Features - Elaboration</t>
+          <t>Warehouse &amp; Inventory Features - Elaboration</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Does your module seamlessly track purchase orders from initial creation all the way through to final invoice payment, as well as maintain comprehensive vendor master records, and also have other relevant features that streamline supplier management?</t>
+          <t>Does your module maintain an inventory master while tracking stock quantities and movements across multiple locations (e.g. warehouses, bins, etc.), optimise supply chain efficiency by automated replenishment, and also have other relevant features that streamline warehouse &amp; inventory management?</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -1657,12 +1673,12 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-21</t>
+          <t>CAT0200-22</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-19-warehouse</t>
+          <t>CAT0200-19-mrp</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -1672,12 +1688,12 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Warehouse &amp; Inventory Features - Elaboration</t>
+          <t>Material Requirements Planning (MRP) Features - Elaboration</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Does your module maintain an inventory master while tracking stock quantities and movements across multiple locations (e.g. warehouses, bins, etc.), optimise supply chain efficiency by automated replenishment, and also have other relevant features that streamline warehouse &amp; inventory management?</t>
+          <t>Does your module dynamically calculate material needs based on demand and supply schedules, automatically trigger purchase requisitions when stock drops below safety-stock thresholds, and also have other relevant features that streamline demand forecasting and inventory reordering?</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -1703,90 +1719,90 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>CAT0200-22</t>
-        </is>
-      </c>
+      <c r="A28" s="2" t="inlineStr"/>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-19-mrp</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>Mandatory</t>
-        </is>
-      </c>
+          <t>CAT0200-13-hr</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr"/>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Material Requirements Planning (MRP) Features - Elaboration</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>Does your module dynamically calculate material needs based on demand and supply schedules, automatically trigger purchase requisitions when stock drops below safety-stock thresholds, and also have other relevant features that streamline demand forecasting and inventory reordering?</t>
-        </is>
-      </c>
+          <t>Human Resources Management Module</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Checkbox</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr"/>
       <c r="H28" s="2" t="inlineStr"/>
       <c r="I28" s="2" t="inlineStr"/>
       <c r="J28" s="2" t="inlineStr"/>
       <c r="K28" s="2" t="inlineStr"/>
       <c r="L28" s="2" t="inlineStr"/>
       <c r="M28" s="2" t="inlineStr"/>
-      <c r="N28" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="N28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr"/>
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>CAT0200-23</t>
+        </is>
+      </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
           <t>CAT0200-13-hr</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr"/>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Human Resources Management Module</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr"/>
+          <t>Human Resource Management System (HRMS) Features</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Do you provide HRMS features?&lt;br/&gt;&lt;br/&gt;**Note:** This sub-module is a **compulsory** requirement of the Human Resources Management Module.</t>
+        </is>
+      </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Label</t>
-        </is>
-      </c>
-      <c r="G29" s="2" t="inlineStr"/>
+          <t>Checkbox</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="H29" s="2" t="inlineStr"/>
       <c r="I29" s="2" t="inlineStr"/>
       <c r="J29" s="2" t="inlineStr"/>
       <c r="K29" s="2" t="inlineStr"/>
       <c r="L29" s="2" t="inlineStr"/>
       <c r="M29" s="2" t="inlineStr"/>
-      <c r="N29" s="2" t="inlineStr"/>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-23</t>
+          <t>CAT0200-24</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-13-hr</t>
+          <t>CAT0200-23-Yes</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -1796,12 +1812,12 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Human Resource Management System (HRMS) Features</t>
+          <t>Human Resource Management System (HRMS) Features - Elaboration</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Do you provide HRMS features?&lt;br/&gt;&lt;br/&gt;**Note:** This sub-module is a **compulsory** requirement of the Human Resources Management Module.</t>
+          <t>Does your module manage personnel master records, payroll processing, leave configurations, and benefits claims while also having other relevant features that facilitate &amp; streamline human resource management systems (HRMS) workflows?</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -1829,7 +1845,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-24</t>
+          <t>CAT0200-25</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -1844,12 +1860,12 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Human Resource Management System (HRMS) Features - Elaboration</t>
+          <t>Finance Module Integration for Payroll</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Does your module manage personnel master records, payroll processing, leave configurations, and benefits claims while also having other relevant features that facilitate &amp; streamline human resource management systems (HRMS) workflows?</t>
+          <t>Is your module integrated with the Finance Management module to facilitate processing of employees' payroll?</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -1877,7 +1893,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-25</t>
+          <t>CAT0200-26</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1892,12 +1908,12 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Finance Module Integration for Payroll</t>
+          <t>IRAS Auto Inclusion Scheme (AIS) Compliance</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Is your module integrated with the Finance Management module to facilitate processing of employees' payroll?</t>
+          <t>Is your solution listed on IRAS's List of Supporting Payroll Software Vendors for the Auto Inclusion Scheme (AIS) for employment income?</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -1925,39 +1941,35 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-26</t>
+          <t>CAT0200-26.1</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-23-Yes</t>
+          <t>CAT0200-13-hr</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Mandatory</t>
+          <t>Preferred</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>IRAS Auto Inclusion Scheme (AIS) Compliance</t>
+          <t>Other Human Resources Sub-Modules</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Is your solution listed on IRAS's List of Supporting Payroll Software Vendors for the Auto Inclusion Scheme (AIS) for employment income?</t>
+          <t>Beyond the mandatory HRMS core, do you provide any other Human Resources sub-modules (such as e-Scheduling, Applicant Tracking &amp; Sourcing, or Employee Rewards and Recognition)?</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Checkbox</t>
-        </is>
-      </c>
-      <c r="G33" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>Radio</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr"/>
       <c r="H33" s="2" t="inlineStr"/>
       <c r="I33" s="2" t="inlineStr"/>
       <c r="J33" s="2" t="inlineStr"/>
@@ -1973,12 +1985,12 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-26.1</t>
+          <t>CAT0200-27</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-13-hr</t>
+          <t>CAT0200-26.1-Yes</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -1988,20 +2000,24 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Other Human Resources Sub-Modules</t>
+          <t>Human Resources Management - Sub-Modules</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Beyond the mandatory HRMS core, do you provide any other Human Resources sub-modules (such as e-Scheduling, Applicant Tracking &amp; Sourcing, or Employee Rewards and Recognition)?</t>
+          <t>Which of these other sub-modules within the Human Resources Management module do you provide?</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Radio</t>
-        </is>
-      </c>
-      <c r="G34" s="2" t="inlineStr"/>
+          <t>Checkbox</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="H34" s="2" t="inlineStr"/>
       <c r="I34" s="2" t="inlineStr"/>
       <c r="J34" s="2" t="inlineStr"/>
@@ -2017,27 +2033,27 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-27</t>
+          <t>CAT0200-28</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-26.1-Yes</t>
+          <t>CAT0200-27-escheduling</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Mandatory</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Human Resources Management - Sub-Modules</t>
+          <t>Human Resource e-Scheduling Features - Elaboration</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Which of these other sub-modules within the Human Resources Management module do you provide?</t>
+          <t>Does your module create employee rosters based on demand and availability, provide mobile cloud access with push notifications for reminders, and also have other relevant features that facilitate &amp; streamline workforce scheduling?</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -2065,12 +2081,12 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-28</t>
+          <t>CAT0200-29</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-27-escheduling</t>
+          <t>CAT0200-27-applicant_tracking</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -2080,12 +2096,12 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Human Resource e-Scheduling Features - Elaboration</t>
+          <t>Applicant Tracking &amp; Sourcing Features - Elaboration</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Does your module create employee rosters based on demand and availability, provide mobile cloud access with push notifications for reminders, and also have other relevant features that facilitate &amp; streamline workforce scheduling?</t>
+          <t>Does your module publish job postings to multiple job boards, track candidate application statuses with customizable communication tools, and also have other relevant features that facilitate &amp; streamline the recruitment and applicant tracking process?</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -2113,12 +2129,12 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-29</t>
+          <t>CAT0200-30</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-27-applicant_tracking</t>
+          <t>CAT0200-27-rewards</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -2128,12 +2144,12 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Applicant Tracking &amp; Sourcing Features - Elaboration</t>
+          <t>Employee Rewards and Recognition Features - Elaboration</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Does your module publish job postings to multiple job boards, track candidate application statuses with customizable communication tools, and also have other relevant features that facilitate &amp; streamline the recruitment and applicant tracking process?</t>
+          <t>Does your module allow employers to award recognition points tied to company values, enable employees to redeem rewards across a diverse network of local merchants, and also have other relevant features that facilitate &amp; streamline employee rewards and appreciation programs?</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -2159,90 +2175,90 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>CAT0200-30</t>
-        </is>
-      </c>
+      <c r="A38" s="2" t="inlineStr"/>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-27-rewards</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>Mandatory</t>
-        </is>
-      </c>
+          <t>CAT0200-13-manufacturing</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr"/>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Employee Rewards and Recognition Features - Elaboration</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>Does your module allow employers to award recognition points tied to company values, enable employees to redeem rewards across a diverse network of local merchants, and also have other relevant features that facilitate &amp; streamline employee rewards and appreciation programs?</t>
-        </is>
-      </c>
+          <t>Manufacturing Management Module</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr"/>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Checkbox</t>
-        </is>
-      </c>
-      <c r="G38" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr"/>
       <c r="H38" s="2" t="inlineStr"/>
       <c r="I38" s="2" t="inlineStr"/>
       <c r="J38" s="2" t="inlineStr"/>
       <c r="K38" s="2" t="inlineStr"/>
       <c r="L38" s="2" t="inlineStr"/>
       <c r="M38" s="2" t="inlineStr"/>
-      <c r="N38" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="N38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr"/>
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>CAT0200-31</t>
+        </is>
+      </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
           <t>CAT0200-13-manufacturing</t>
         </is>
       </c>
-      <c r="C39" s="2" t="inlineStr"/>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Manufacturing Management Module</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr"/>
+          <t>Manufacturing Management - Sub-Modules</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Which of these sub-modules within the Manufacturing Management module do you provide?&lt;br/&gt;&lt;br/&gt;**Note:** You have to select at least 1 option to qualify for this module.</t>
+        </is>
+      </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Label</t>
-        </is>
-      </c>
-      <c r="G39" s="2" t="inlineStr"/>
+          <t>Checkbox</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="H39" s="2" t="inlineStr"/>
       <c r="I39" s="2" t="inlineStr"/>
       <c r="J39" s="2" t="inlineStr"/>
       <c r="K39" s="2" t="inlineStr"/>
       <c r="L39" s="2" t="inlineStr"/>
       <c r="M39" s="2" t="inlineStr"/>
-      <c r="N39" s="2" t="inlineStr"/>
+      <c r="N39" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-31</t>
+          <t>CAT0200-32</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-13-manufacturing</t>
+          <t>CAT0200-31-mes</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -2252,12 +2268,12 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Manufacturing Management - Sub-Modules</t>
+          <t>Manufacturing Execution System (MES) Features</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Which of these sub-modules within the Manufacturing Management module do you provide?&lt;br/&gt;&lt;br/&gt;**Note:** You have to select at least 1 option to qualify for this module.</t>
+          <t>Does your module create, dispatch, and plan work order sequences across shopfloor stations, generate comprehensive MES dashboards and reports for key production indicators, and also have other relevant features that facilitate &amp; streamline manufacturing execution and work order management?</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -2285,7 +2301,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-32</t>
+          <t>CAT0200-33</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -2295,29 +2311,25 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Mandatory</t>
+          <t>Preferred</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Manufacturing Execution System (MES) Features</t>
+          <t>MES Shopfloor Data Collection Features (Manual)</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Does your module create, dispatch, and plan work order sequences across shopfloor stations, generate comprehensive MES dashboards and reports for key production indicators, and also have other relevant features that facilitate &amp; streamline manufacturing execution and work order management?</t>
+          <t>Does your module enable operators to view detailed task information and input production data on the shopfloor, track and display real-time work-in-progress (WIP) status for each operation, and also have other relevant features that facilitate &amp; streamline shopfloor tracking and data collection?</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Checkbox</t>
-        </is>
-      </c>
-      <c r="G41" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>Radio</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr"/>
       <c r="H41" s="2" t="inlineStr"/>
       <c r="I41" s="2" t="inlineStr"/>
       <c r="J41" s="2" t="inlineStr"/>
@@ -2333,7 +2345,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-33</t>
+          <t>CAT0200-34</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -2348,12 +2360,12 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>MES Shopfloor Data Collection Features (Manual)</t>
+          <t>MES Shopfloor Data Collection Features (Automated)</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Does your module enable operators to view detailed task information and input production data on the shopfloor, track and display real-time work-in-progress (WIP) status for each operation, and also have other relevant features that facilitate &amp; streamline shopfloor tracking and data collection?</t>
+          <t>Does your module monitor real-time equipment status, maintain equipment data, and track shopfloor data entry alongside work-in-progress (WIP) statuses, and also have other relevant features that facilitate &amp; streamline equipment monitoring and shopfloor tracking?</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -2377,35 +2389,39 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-34</t>
+          <t>CAT0200-35</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-31-mes</t>
+          <t>CAT0200-31-qm</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Mandatory</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>MES Shopfloor Data Collection Features (Automated)</t>
+          <t>Quality Management (QM) Features</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Does your module monitor real-time equipment status, maintain equipment data, and track shopfloor data entry alongside work-in-progress (WIP) statuses, and also have other relevant features that facilitate &amp; streamline equipment monitoring and shopfloor tracking?</t>
+          <t>Does your module configure quality inspection plans, collect measurement data manually or via equipment integration, and automatically trigger non-conformance alerts with root cause recording, and also have other relevant features that facilitate &amp; streamline quality management workflows?</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Radio</t>
-        </is>
-      </c>
-      <c r="G43" s="2" t="inlineStr"/>
+          <t>Checkbox</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="H43" s="2" t="inlineStr"/>
       <c r="I43" s="2" t="inlineStr"/>
       <c r="J43" s="2" t="inlineStr"/>
@@ -2421,12 +2437,12 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-35</t>
+          <t>CAT0200-36</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-31-qm</t>
+          <t>CAT0200-31-plm</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -2436,12 +2452,12 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Quality Management (QM) Features</t>
+          <t>Product Lifecycle Management (PLM) Features</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Does your module configure quality inspection plans, collect measurement data manually or via equipment integration, and automatically trigger non-conformance alerts with root cause recording, and also have other relevant features that facilitate &amp; streamline quality management workflows?</t>
+          <t>Does your module centralise routing and work instructions (including engineering drawing, tool, and manpower management) while governing revisions through engineering change management, and also have other relevant features that facilitate &amp; streamline product lifecycle management (PLM) workflows?</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -2467,85 +2483,85 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>CAT0200-36</t>
-        </is>
-      </c>
+      <c r="A45" s="2" t="inlineStr"/>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-31-plm</t>
-        </is>
-      </c>
-      <c r="C45" s="2" t="inlineStr">
-        <is>
-          <t>Mandatory</t>
-        </is>
-      </c>
+          <t>CAT0200-13-fleet</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr"/>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Product Lifecycle Management (PLM) Features</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr">
-        <is>
-          <t>Does your module centralise routing and work instructions (including engineering drawing, tool, and manpower management) while governing revisions through engineering change management, and also have other relevant features that facilitate &amp; streamline product lifecycle management (PLM) workflows?</t>
-        </is>
-      </c>
+          <t>Fleet Management Module</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr"/>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Checkbox</t>
-        </is>
-      </c>
-      <c r="G45" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr"/>
       <c r="H45" s="2" t="inlineStr"/>
       <c r="I45" s="2" t="inlineStr"/>
       <c r="J45" s="2" t="inlineStr"/>
       <c r="K45" s="2" t="inlineStr"/>
       <c r="L45" s="2" t="inlineStr"/>
       <c r="M45" s="2" t="inlineStr"/>
-      <c r="N45" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="N45" s="2" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="inlineStr"/>
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>CAT0200-37</t>
+        </is>
+      </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
           <t>CAT0200-13-fleet</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr"/>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Fleet Management Module</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr"/>
+          <t>Fleet Management Module Features</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Does your module use telematics and GPS for real-time fleet tracking, automate dispatch and dynamic route planning using live traffic data, and also have other relevant features that facilitate &amp; streamline fleet management and transport operations?</t>
+        </is>
+      </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Label</t>
-        </is>
-      </c>
-      <c r="G46" s="2" t="inlineStr"/>
+          <t>Checkbox</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="H46" s="2" t="inlineStr"/>
       <c r="I46" s="2" t="inlineStr"/>
       <c r="J46" s="2" t="inlineStr"/>
       <c r="K46" s="2" t="inlineStr"/>
       <c r="L46" s="2" t="inlineStr"/>
       <c r="M46" s="2" t="inlineStr"/>
-      <c r="N46" s="2" t="inlineStr"/>
+      <c r="N46" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-37</t>
+          <t>CAT0200-38</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -2555,29 +2571,25 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Mandatory</t>
+          <t>Preferred</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Fleet Management Module Features</t>
+          <t>Fleet Management Module Safety Features</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Does your module use telematics and GPS for real-time fleet tracking, automate dispatch and dynamic route planning using live traffic data, and also have other relevant features that facilitate &amp; streamline fleet management and transport operations?</t>
+          <t>Does your module monitor driver status to detect fatigue or distractions, provide advanced driver assistance warnings for potential collisions, and also have other relevant features that facilitate &amp; streamline driver safety?</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Checkbox</t>
-        </is>
-      </c>
-      <c r="G47" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>Radio</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr"/>
       <c r="H47" s="2" t="inlineStr"/>
       <c r="I47" s="2" t="inlineStr"/>
       <c r="J47" s="2" t="inlineStr"/>
@@ -2591,34 +2603,22 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>CAT0200-38</t>
-        </is>
-      </c>
+      <c r="A48" s="2" t="inlineStr"/>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-13-fleet</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>Preferred</t>
-        </is>
-      </c>
+          <t>CAT0200-13-field_service</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr"/>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Fleet Management Module Safety Features</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>Does your module monitor driver status to detect fatigue or distractions, provide advanced driver assistance warnings for potential collisions, and also have other relevant features that facilitate &amp; streamline driver safety?</t>
-        </is>
-      </c>
+          <t>Field Service Management Module</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr"/>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>Radio</t>
+          <t>Label</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr"/>
@@ -2628,257 +2628,257 @@
       <c r="K48" s="2" t="inlineStr"/>
       <c r="L48" s="2" t="inlineStr"/>
       <c r="M48" s="2" t="inlineStr"/>
-      <c r="N48" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="N48" s="2" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="inlineStr"/>
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>CAT0200-39</t>
+        </is>
+      </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
           <t>CAT0200-13-field_service</t>
         </is>
       </c>
-      <c r="C49" s="2" t="inlineStr"/>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Field Service Management Module</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="inlineStr"/>
+          <t>Field Service Management (FSM) Module Features</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>Does your module create, assign, and allow the scheduling of work orders based on technician profiles, offer a mobile app for field workers to update job statuses with digital proof, and also have other relevant features that facilitate &amp; streamline field service management (FSM) workflows?</t>
+        </is>
+      </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Label</t>
-        </is>
-      </c>
-      <c r="G49" s="2" t="inlineStr"/>
+          <t>Checkbox</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="H49" s="2" t="inlineStr"/>
       <c r="I49" s="2" t="inlineStr"/>
       <c r="J49" s="2" t="inlineStr"/>
       <c r="K49" s="2" t="inlineStr"/>
       <c r="L49" s="2" t="inlineStr"/>
       <c r="M49" s="2" t="inlineStr"/>
-      <c r="N49" s="2" t="inlineStr"/>
+      <c r="N49" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>CAT0200-39</t>
-        </is>
-      </c>
+      <c r="A50" s="2" t="inlineStr"/>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-13-field_service</t>
-        </is>
-      </c>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t>Mandatory</t>
-        </is>
-      </c>
+          <t>CAT0200-13-project</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr"/>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Field Service Management (FSM) Module Features</t>
-        </is>
-      </c>
-      <c r="E50" s="2" t="inlineStr">
-        <is>
-          <t>Does your module create, assign, and allow the scheduling of work orders based on technician profiles, offer a mobile app for field workers to update job statuses with digital proof, and also have other relevant features that facilitate &amp; streamline field service management (FSM) workflows?</t>
-        </is>
-      </c>
+          <t>Project Management Module</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr"/>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>Checkbox</t>
-        </is>
-      </c>
-      <c r="G50" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr"/>
       <c r="H50" s="2" t="inlineStr"/>
       <c r="I50" s="2" t="inlineStr"/>
       <c r="J50" s="2" t="inlineStr"/>
       <c r="K50" s="2" t="inlineStr"/>
       <c r="L50" s="2" t="inlineStr"/>
       <c r="M50" s="2" t="inlineStr"/>
-      <c r="N50" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="N50" s="2" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="inlineStr"/>
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>CAT0200-40</t>
+        </is>
+      </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
           <t>CAT0200-13-project</t>
         </is>
       </c>
-      <c r="C51" s="2" t="inlineStr"/>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Project Management Module</t>
-        </is>
-      </c>
-      <c r="E51" s="2" t="inlineStr"/>
+          <t>Project Management (PM) Module Features</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>Does your module manage and schedule project tasks with clear deadlines and dependencies, track team workloads and resource allocation, and also have other relevant features that facilitate &amp; streamline the project management (PM) process?</t>
+        </is>
+      </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Label</t>
-        </is>
-      </c>
-      <c r="G51" s="2" t="inlineStr"/>
+          <t>Checkbox</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="H51" s="2" t="inlineStr"/>
       <c r="I51" s="2" t="inlineStr"/>
       <c r="J51" s="2" t="inlineStr"/>
       <c r="K51" s="2" t="inlineStr"/>
       <c r="L51" s="2" t="inlineStr"/>
       <c r="M51" s="2" t="inlineStr"/>
-      <c r="N51" s="2" t="inlineStr"/>
+      <c r="N51" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t>CAT0200-40</t>
-        </is>
-      </c>
+      <c r="A52" s="2" t="inlineStr"/>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-13-project</t>
-        </is>
-      </c>
-      <c r="C52" s="2" t="inlineStr">
-        <is>
-          <t>Mandatory</t>
-        </is>
-      </c>
+          <t>CAT0200-13-asset</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr"/>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Project Management (PM) Module Features</t>
-        </is>
-      </c>
-      <c r="E52" s="2" t="inlineStr">
-        <is>
-          <t>Does your module manage and schedule project tasks with clear deadlines and dependencies, track team workloads and resource allocation, and also have other relevant features that facilitate &amp; streamline the project management (PM) process?</t>
-        </is>
-      </c>
+          <t>Asset Management Module</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr"/>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Checkbox</t>
-        </is>
-      </c>
-      <c r="G52" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr"/>
       <c r="H52" s="2" t="inlineStr"/>
       <c r="I52" s="2" t="inlineStr"/>
       <c r="J52" s="2" t="inlineStr"/>
       <c r="K52" s="2" t="inlineStr"/>
       <c r="L52" s="2" t="inlineStr"/>
       <c r="M52" s="2" t="inlineStr"/>
-      <c r="N52" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="N52" s="2" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="inlineStr"/>
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>CAT0200-41</t>
+        </is>
+      </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
           <t>CAT0200-13-asset</t>
         </is>
       </c>
-      <c r="C53" s="2" t="inlineStr"/>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Asset Management Module</t>
-        </is>
-      </c>
-      <c r="E53" s="2" t="inlineStr"/>
+          <t>Asset Management Module Features</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>Does your module track the centralised lifecycle of assets from procurement to decommissioning, automate maintenance scheduling based on usage thresholds, and continuously monitor equipment utilisation and compliance histories across multiple sites, and also have other relevant features that facilitate &amp; streamline asset management?</t>
+        </is>
+      </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>Label</t>
-        </is>
-      </c>
-      <c r="G53" s="2" t="inlineStr"/>
+          <t>Checkbox</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="H53" s="2" t="inlineStr"/>
       <c r="I53" s="2" t="inlineStr"/>
       <c r="J53" s="2" t="inlineStr"/>
       <c r="K53" s="2" t="inlineStr"/>
       <c r="L53" s="2" t="inlineStr"/>
       <c r="M53" s="2" t="inlineStr"/>
-      <c r="N53" s="2" t="inlineStr"/>
+      <c r="N53" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>CAT0200-41</t>
-        </is>
-      </c>
-      <c r="B54" s="2" t="inlineStr">
-        <is>
-          <t>CAT0200-13-asset</t>
-        </is>
-      </c>
-      <c r="C54" s="2" t="inlineStr">
-        <is>
-          <t>Mandatory</t>
-        </is>
-      </c>
+      <c r="A54" s="2" t="inlineStr"/>
+      <c r="B54" s="2" t="inlineStr"/>
+      <c r="C54" s="2" t="inlineStr"/>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Asset Management Module Features</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="inlineStr">
-        <is>
-          <t>Does your module track the centralised lifecycle of assets from procurement to decommissioning, automate maintenance scheduling based on usage thresholds, and continuously monitor equipment utilisation and compliance histories across multiple sites, and also have other relevant features that facilitate &amp; streamline asset management?</t>
-        </is>
-      </c>
+          <t>Others Module</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr"/>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Checkbox</t>
-        </is>
-      </c>
-      <c r="G54" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr"/>
       <c r="H54" s="2" t="inlineStr"/>
       <c r="I54" s="2" t="inlineStr"/>
       <c r="J54" s="2" t="inlineStr"/>
       <c r="K54" s="2" t="inlineStr"/>
       <c r="L54" s="2" t="inlineStr"/>
       <c r="M54" s="2" t="inlineStr"/>
-      <c r="N54" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="N54" s="2" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="inlineStr"/>
-      <c r="B55" s="2" t="inlineStr">
-        <is>
-          <t>CAT0200-13.1-Yes</t>
-        </is>
-      </c>
-      <c r="C55" s="2" t="inlineStr"/>
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>CAT0200-13.1</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr"/>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Preferred</t>
+        </is>
+      </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
           <t>Others Module</t>
         </is>
       </c>
-      <c r="E55" s="2" t="inlineStr"/>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>Do you also provide an ERP module that is not covered by the list above (an "Others" module)?&lt;br/&gt;&lt;br/&gt;You may submit at most 1 "Others" module, and it does not count toward the minimum of 3 modules above. Select "Yes" to declare it below.</t>
+        </is>
+      </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Label</t>
+          <t>Radio</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr"/>
@@ -2888,7 +2888,11 @@
       <c r="K55" s="2" t="inlineStr"/>
       <c r="L55" s="2" t="inlineStr"/>
       <c r="M55" s="2" t="inlineStr"/>
-      <c r="N55" s="2" t="inlineStr"/>
+      <c r="N55" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -5481,12 +5485,12 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-13.1</t>
+          <t>CAT0200-14</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-13.1-Yes</t>
+          <t>CAT0200-14-Yes</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -5499,17 +5503,17 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-13.1</t>
+          <t>CAT0200-15</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-13.1-No</t>
+          <t>CAT0200-15-Yes</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr"/>
@@ -5517,17 +5521,17 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-14</t>
+          <t>CAT0200-16</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-14-Yes</t>
+          <t>CAT0200-16-sales</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr"/>
@@ -5535,17 +5539,17 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-15</t>
+          <t>CAT0200-16</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-15-Yes</t>
+          <t>CAT0200-16-crm</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Customer Relationship Management (CRM)</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr"/>
@@ -5553,17 +5557,17 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-16</t>
+          <t>CAT0200-17</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-16-sales</t>
+          <t>CAT0200-17-Yes</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr"/>
@@ -5571,17 +5575,17 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-16</t>
+          <t>CAT0200-18</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-16-crm</t>
+          <t>CAT0200-18-Yes</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Customer Relationship Management (CRM)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr"/>
@@ -5589,17 +5593,17 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-17</t>
+          <t>CAT0200-19</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-17-Yes</t>
+          <t>CAT0200-19-procurement</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Procurement &amp; Purchasing</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr"/>
@@ -5607,17 +5611,17 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-18</t>
+          <t>CAT0200-19</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-18-Yes</t>
+          <t>CAT0200-19-warehouse</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Warehouse &amp; Inventory</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr"/>
@@ -5630,12 +5634,12 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-19-procurement</t>
+          <t>CAT0200-19-mrp</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Procurement &amp; Purchasing</t>
+          <t>Material Requirements Planning (MRP)</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr"/>
@@ -5643,17 +5647,17 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-19</t>
+          <t>CAT0200-20</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-19-warehouse</t>
+          <t>CAT0200-20-Yes</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Warehouse &amp; Inventory</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr"/>
@@ -5661,17 +5665,17 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-19</t>
+          <t>CAT0200-21</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-19-mrp</t>
+          <t>CAT0200-21-Yes</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Material Requirements Planning (MRP)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr"/>
@@ -5679,12 +5683,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-20</t>
+          <t>CAT0200-22</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-20-Yes</t>
+          <t>CAT0200-22-Yes</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -5697,12 +5701,12 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-21</t>
+          <t>CAT0200-23</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-21-Yes</t>
+          <t>CAT0200-23-Yes</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -5715,12 +5719,12 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-22</t>
+          <t>CAT0200-24</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-22-Yes</t>
+          <t>CAT0200-24-Yes</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -5733,12 +5737,12 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-23</t>
+          <t>CAT0200-25</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-23-Yes</t>
+          <t>CAT0200-25-Yes</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -5751,12 +5755,12 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-24</t>
+          <t>CAT0200-26</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-24-Yes</t>
+          <t>CAT0200-26-Yes</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -5769,12 +5773,12 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-25</t>
+          <t>CAT0200-26.1</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-25-Yes</t>
+          <t>CAT0200-26.1-Yes</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -5787,17 +5791,17 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-26</t>
+          <t>CAT0200-26.1</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-26-Yes</t>
+          <t>CAT0200-26.1-No</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr"/>
@@ -5805,17 +5809,17 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-26.1</t>
+          <t>CAT0200-27</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-26.1-Yes</t>
+          <t>CAT0200-27-escheduling</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Human Resource e-Scheduling</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr"/>
@@ -5823,17 +5827,17 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-26.1</t>
+          <t>CAT0200-27</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-26.1-No</t>
+          <t>CAT0200-27-applicant_tracking</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Applicant Tracking &amp; Sourcing</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr"/>
@@ -5846,12 +5850,12 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-27-escheduling</t>
+          <t>CAT0200-27-rewards</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Human Resource e-Scheduling</t>
+          <t>Employee Rewards and Recognition</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr"/>
@@ -5859,17 +5863,17 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-27</t>
+          <t>CAT0200-28</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-27-applicant_tracking</t>
+          <t>CAT0200-28-Yes</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Applicant Tracking &amp; Sourcing</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr"/>
@@ -5877,17 +5881,17 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-27</t>
+          <t>CAT0200-29</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-27-rewards</t>
+          <t>CAT0200-29-Yes</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Employee Rewards and Recognition</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr"/>
@@ -5895,12 +5899,12 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-28</t>
+          <t>CAT0200-30</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-28-Yes</t>
+          <t>CAT0200-30-Yes</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -5913,17 +5917,17 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-29</t>
+          <t>CAT0200-31</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-29-Yes</t>
+          <t>CAT0200-31-mes</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Manufacturing Execution System (MES)</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr"/>
@@ -5931,17 +5935,17 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-30</t>
+          <t>CAT0200-31</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-30-Yes</t>
+          <t>CAT0200-31-qm</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Quality Management (QM)</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr"/>
@@ -5954,12 +5958,12 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-31-mes</t>
+          <t>CAT0200-31-plm</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Manufacturing Execution System (MES)</t>
+          <t>Product Lifecycle Management (PLM)</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr"/>
@@ -5967,17 +5971,17 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-31</t>
+          <t>CAT0200-32</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-31-qm</t>
+          <t>CAT0200-32-Yes</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Quality Management (QM)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr"/>
@@ -5985,17 +5989,17 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-31</t>
+          <t>CAT0200-33</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-31-plm</t>
+          <t>CAT0200-33-Yes</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Product Lifecycle Management (PLM)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr"/>
@@ -6003,17 +6007,17 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-32</t>
+          <t>CAT0200-33</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-32-Yes</t>
+          <t>CAT0200-33-No</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr"/>
@@ -6021,12 +6025,12 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-33</t>
+          <t>CAT0200-34</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-33-Yes</t>
+          <t>CAT0200-34-Yes</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -6039,12 +6043,12 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-33</t>
+          <t>CAT0200-34</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-33-No</t>
+          <t>CAT0200-34-No</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -6057,12 +6061,12 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-34</t>
+          <t>CAT0200-35</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-34-Yes</t>
+          <t>CAT0200-35-Yes</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
@@ -6075,17 +6079,17 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-34</t>
+          <t>CAT0200-36</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-34-No</t>
+          <t>CAT0200-36-Yes</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr"/>
@@ -6093,12 +6097,12 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-35</t>
+          <t>CAT0200-37</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-35-Yes</t>
+          <t>CAT0200-37-Yes</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
@@ -6111,12 +6115,12 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-36</t>
+          <t>CAT0200-38</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-36-Yes</t>
+          <t>CAT0200-38-Yes</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -6129,17 +6133,17 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-37</t>
+          <t>CAT0200-38</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-37-Yes</t>
+          <t>CAT0200-38-No</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr"/>
@@ -6147,12 +6151,12 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-38</t>
+          <t>CAT0200-39</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-38-Yes</t>
+          <t>CAT0200-39-Yes</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
@@ -6165,17 +6169,17 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-38</t>
+          <t>CAT0200-40</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-38-No</t>
+          <t>CAT0200-40-Yes</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr"/>
@@ -6183,12 +6187,12 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-39</t>
+          <t>CAT0200-41</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-39-Yes</t>
+          <t>CAT0200-41-Yes</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
@@ -6201,12 +6205,12 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-40</t>
+          <t>CAT0200-13.1</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-40-Yes</t>
+          <t>CAT0200-13.1-Yes</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
@@ -6219,17 +6223,17 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-41</t>
+          <t>CAT0200-13.1</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-41-Yes</t>
+          <t>CAT0200-13.1-No</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Declaration 'above'->'below'; trim Q13 wording + drop Others note; republish xlsx
</commit_message>
<xml_diff>
--- a/cat0200_import.xlsx
+++ b/cat0200_import.xlsx
@@ -1177,7 +1177,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Which ERP modules does your solution provide?&lt;br/&gt;&lt;br/&gt;Please select a minimum of at least 3 modules.&lt;br/&gt;&lt;br/&gt;**Note:** To submit an additional module not covered in the list above, use the "Others Module" question shown after the module sections. "Others" does not count toward the minimum of 3 modules.</t>
+          <t>Which ERP modules does your solution provide?&lt;br/&gt;&lt;br/&gt;Please select at least 3 modules.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -3401,7 +3401,7 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Which third-party ERP module/application types can your solution integrate with?&lt;br/&gt;&lt;br/&gt;Please select a minimum of at least 1 module.&lt;br/&gt;&lt;br/&gt;**Note 1:** You can only be qualified for up to the 9 modules defined above. Submissions for other undefined modules not in the list will not be accepted.</t>
+          <t>Which third-party ERP module/application types can your solution integrate with?&lt;br/&gt;&lt;br/&gt;Please select at least 1 module.&lt;br/&gt;&lt;br/&gt;**Note 1:** You can only be qualified for up to the 9 modules defined above. Submissions for other undefined modules not in the list will not be accepted.</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
@@ -5315,7 +5315,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>I confirm I have completed the instruction(s) and provided the information above.</t>
+          <t>I confirm I have completed the instruction(s) and provided the information below.</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr"/>
@@ -6251,7 +6251,7 @@
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>I confirm I have completed the instruction(s) and provided the information above.</t>
+          <t>I confirm I have completed the instruction(s) and provided the information below.</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr"/>
@@ -6269,7 +6269,7 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>I confirm I have completed the instruction(s) and provided the information above.</t>
+          <t>I confirm I have completed the instruction(s) and provided the information below.</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr"/>
@@ -7799,7 +7799,7 @@
       </c>
       <c r="C159" s="2" t="inlineStr">
         <is>
-          <t>I confirm I have completed the instruction(s) and provided the information above.</t>
+          <t>I confirm I have completed the instruction(s) and provided the information below.</t>
         </is>
       </c>
       <c r="D159" s="2" t="inlineStr"/>
@@ -7817,7 +7817,7 @@
       </c>
       <c r="C160" s="2" t="inlineStr">
         <is>
-          <t>I confirm I have completed the instruction(s) and provided the information above.</t>
+          <t>I confirm I have completed the instruction(s) and provided the information below.</t>
         </is>
       </c>
       <c r="D160" s="2" t="inlineStr"/>
@@ -7853,7 +7853,7 @@
       </c>
       <c r="C162" s="2" t="inlineStr">
         <is>
-          <t>I confirm I have completed the instruction(s) and provided the information above.</t>
+          <t>I confirm I have completed the instruction(s) and provided the information below.</t>
         </is>
       </c>
       <c r="D162" s="2" t="inlineStr"/>
@@ -7871,7 +7871,7 @@
       </c>
       <c r="C163" s="2" t="inlineStr">
         <is>
-          <t>I confirm I have completed the instruction(s) and provided the information above.</t>
+          <t>I confirm I have completed the instruction(s) and provided the information below.</t>
         </is>
       </c>
       <c r="D163" s="2" t="inlineStr"/>
@@ -7907,7 +7907,7 @@
       </c>
       <c r="C165" s="2" t="inlineStr">
         <is>
-          <t>I confirm I have completed the instruction(s) and provided the information above.</t>
+          <t>I confirm I have completed the instruction(s) and provided the information below.</t>
         </is>
       </c>
       <c r="D165" s="2" t="inlineStr"/>
@@ -7925,7 +7925,7 @@
       </c>
       <c r="C166" s="2" t="inlineStr">
         <is>
-          <t>I confirm I have completed the instruction(s) and provided the information above.</t>
+          <t>I confirm I have completed the instruction(s) and provided the information below.</t>
         </is>
       </c>
       <c r="D166" s="2" t="inlineStr"/>
@@ -7961,7 +7961,7 @@
       </c>
       <c r="C168" s="2" t="inlineStr">
         <is>
-          <t>I confirm I have completed the instruction(s) and provided the information above.</t>
+          <t>I confirm I have completed the instruction(s) and provided the information below.</t>
         </is>
       </c>
       <c r="D168" s="2" t="inlineStr"/>
@@ -7979,7 +7979,7 @@
       </c>
       <c r="C169" s="2" t="inlineStr">
         <is>
-          <t>I confirm I have completed the instruction(s) and provided the information above.</t>
+          <t>I confirm I have completed the instruction(s) and provided the information below.</t>
         </is>
       </c>
       <c r="D169" s="2" t="inlineStr"/>
@@ -8015,7 +8015,7 @@
       </c>
       <c r="C171" s="2" t="inlineStr">
         <is>
-          <t>I confirm I have completed the instruction(s) and provided the information above.</t>
+          <t>I confirm I have completed the instruction(s) and provided the information below.</t>
         </is>
       </c>
       <c r="D171" s="2" t="inlineStr"/>
@@ -8033,7 +8033,7 @@
       </c>
       <c r="C172" s="2" t="inlineStr">
         <is>
-          <t>I confirm I have completed the instruction(s) and provided the information above.</t>
+          <t>I confirm I have completed the instruction(s) and provided the information below.</t>
         </is>
       </c>
       <c r="D172" s="2" t="inlineStr"/>
@@ -8069,7 +8069,7 @@
       </c>
       <c r="C174" s="2" t="inlineStr">
         <is>
-          <t>I confirm I have completed the instruction(s) and provided the information above.</t>
+          <t>I confirm I have completed the instruction(s) and provided the information below.</t>
         </is>
       </c>
       <c r="D174" s="2" t="inlineStr"/>
@@ -8087,7 +8087,7 @@
       </c>
       <c r="C175" s="2" t="inlineStr">
         <is>
-          <t>I confirm I have completed the instruction(s) and provided the information above.</t>
+          <t>I confirm I have completed the instruction(s) and provided the information below.</t>
         </is>
       </c>
       <c r="D175" s="2" t="inlineStr"/>
@@ -8123,7 +8123,7 @@
       </c>
       <c r="C177" s="2" t="inlineStr">
         <is>
-          <t>I confirm I have completed the instruction(s) and provided the information above.</t>
+          <t>I confirm I have completed the instruction(s) and provided the information below.</t>
         </is>
       </c>
       <c r="D177" s="2" t="inlineStr"/>
@@ -8141,7 +8141,7 @@
       </c>
       <c r="C178" s="2" t="inlineStr">
         <is>
-          <t>I confirm I have completed the instruction(s) and provided the information above.</t>
+          <t>I confirm I have completed the instruction(s) and provided the information below.</t>
         </is>
       </c>
       <c r="D178" s="2" t="inlineStr"/>
@@ -8177,7 +8177,7 @@
       </c>
       <c r="C180" s="2" t="inlineStr">
         <is>
-          <t>I confirm I have completed the instruction(s) and provided the information above.</t>
+          <t>I confirm I have completed the instruction(s) and provided the information below.</t>
         </is>
       </c>
       <c r="D180" s="2" t="inlineStr"/>
@@ -8195,7 +8195,7 @@
       </c>
       <c r="C181" s="2" t="inlineStr">
         <is>
-          <t>I confirm I have completed the instruction(s) and provided the information above.</t>
+          <t>I confirm I have completed the instruction(s) and provided the information below.</t>
         </is>
       </c>
       <c r="D181" s="2" t="inlineStr"/>
@@ -8231,7 +8231,7 @@
       </c>
       <c r="C183" s="2" t="inlineStr">
         <is>
-          <t>I confirm I have completed the instruction(s) and provided the information above.</t>
+          <t>I confirm I have completed the instruction(s) and provided the information below.</t>
         </is>
       </c>
       <c r="D183" s="2" t="inlineStr"/>
@@ -8249,7 +8249,7 @@
       </c>
       <c r="C184" s="2" t="inlineStr">
         <is>
-          <t>I confirm I have completed the instruction(s) and provided the information above.</t>
+          <t>I confirm I have completed the instruction(s) and provided the information below.</t>
         </is>
       </c>
       <c r="D184" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Renumber Others opt-in 13.1 -> 41.1 (IDs sort into display order); republish xlsx
</commit_message>
<xml_diff>
--- a/cat0200_import.xlsx
+++ b/cat0200_import.xlsx
@@ -2857,7 +2857,7 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-13.1</t>
+          <t>CAT0200-41.1</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr"/>
@@ -2902,7 +2902,7 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-13.1-Yes</t>
+          <t>CAT0200-41.1-Yes</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -2958,7 +2958,7 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-13.1-Yes</t>
+          <t>CAT0200-41.1-Yes</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -3022,7 +3022,7 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-13.1-Yes</t>
+          <t>CAT0200-41.1-Yes</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -3078,7 +3078,7 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-13.1-Yes</t>
+          <t>CAT0200-41.1-Yes</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -3122,7 +3122,7 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-13.1-Yes</t>
+          <t>CAT0200-41.1-Yes</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -3178,7 +3178,7 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-13.1-Yes</t>
+          <t>CAT0200-41.1-Yes</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -3222,7 +3222,7 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-13.1-Yes</t>
+          <t>CAT0200-41.1-Yes</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -3278,7 +3278,7 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-13.1-Yes</t>
+          <t>CAT0200-41.1-Yes</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
@@ -6205,12 +6205,12 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-13.1</t>
+          <t>CAT0200-41.1</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-13.1-Yes</t>
+          <t>CAT0200-41.1-Yes</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
@@ -6223,12 +6223,12 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-13.1</t>
+          <t>CAT0200-41.1</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>CAT0200-13.1-No</t>
+          <t>CAT0200-41.1-No</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Q51 note 'above'->'listed below'; reword 3 Others proposal asks; republish xlsx
</commit_message>
<xml_diff>
--- a/cat0200_import.xlsx
+++ b/cat0200_import.xlsx
@@ -3037,7 +3037,7 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Please submit 1st of 3 completed project proposals that include the following, in 1 continuous PDF document:&lt;br/&gt;&lt;br/&gt;1) Proof of Implementation for the Submitted Module&lt;br/&gt;2) Project Completion Signoff Proof by Client&lt;br/&gt;3) Project Completion Date&lt;br/&gt;4) Total Overall Billed Costs</t>
+          <t>Please submit your 1st completed project proposal as one continuous PDF document, including the following:&lt;br/&gt;&lt;br/&gt;1) Proof of Implementation for the Submitted Module&lt;br/&gt;2) Project Completion Signoff Proof by Client&lt;br/&gt;3) Project Completion Date&lt;br/&gt;4) Total Overall Billed Costs</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
@@ -3137,7 +3137,7 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Please submit 2nd of 3 completed project proposals that include the following, in 1 continuous PDF document:&lt;br/&gt;&lt;br/&gt;1) Proof of Implementation for the Submitted Module&lt;br/&gt;2) Project Completion Signoff Proof by Client&lt;br/&gt;3) Project Completion Date&lt;br/&gt;4) Total Overall Billed Costs</t>
+          <t>Please submit your 2nd completed project proposal as one continuous PDF document, including the following:&lt;br/&gt;&lt;br/&gt;1) Proof of Implementation for the Submitted Module&lt;br/&gt;2) Project Completion Signoff Proof by Client&lt;br/&gt;3) Project Completion Date&lt;br/&gt;4) Total Overall Billed Costs</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
@@ -3237,7 +3237,7 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Please submit 3rd of 3 completed project proposals that include the following, in 1 continuous PDF document:&lt;br/&gt;&lt;br/&gt;1) Proof of Implementation for the Submitted Module&lt;br/&gt;2) Project Completion Signoff Proof by Client&lt;br/&gt;3) Project Completion Date&lt;br/&gt;4) Total Overall Billed Costs</t>
+          <t>Please submit your 3rd completed project proposal as one continuous PDF document, including the following:&lt;br/&gt;&lt;br/&gt;1) Proof of Implementation for the Submitted Module&lt;br/&gt;2) Project Completion Signoff Proof by Client&lt;br/&gt;3) Project Completion Date&lt;br/&gt;4) Total Overall Billed Costs</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
@@ -3401,7 +3401,7 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Which third-party ERP module/application types can your solution integrate with?&lt;br/&gt;&lt;br/&gt;Please select at least 1 module.&lt;br/&gt;&lt;br/&gt;**Note 1:** You can only be qualified for up to the 9 modules defined above. Submissions for other undefined modules not in the list will not be accepted.</t>
+          <t>Which third-party ERP module/application types can your solution integrate with?&lt;br/&gt;&lt;br/&gt;Please select at least 1 module.&lt;br/&gt;&lt;br/&gt;**Note 1:** You can only be qualified for up to the 9 modules listed below. Submissions for other undefined modules not in the list will not be accepted.</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Others evidence titles: add /3 stage marker; republish xlsx
</commit_message>
<xml_diff>
--- a/cat0200_import.xlsx
+++ b/cat0200_import.xlsx
@@ -3032,7 +3032,7 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>"Others" Module Evidence 1</t>
+          <t>"Others" Module Evidence 1/3</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>"Others" Module Evidence 1 - Client's Sector</t>
+          <t>"Others" Module Evidence 1/3 - Client's Sector</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
@@ -3132,7 +3132,7 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>"Others" Module Evidence 2</t>
+          <t>"Others" Module Evidence 2/3</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -3188,7 +3188,7 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>"Others" Module Evidence 2 - Client's Sector</t>
+          <t>"Others" Module Evidence 2/3 - Client's Sector</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
@@ -3232,7 +3232,7 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>"Others" Module Evidence 3</t>
+          <t>"Others" Module Evidence 3/3</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -3288,7 +3288,7 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>"Others" Module Evidence 3 - Client's Sector</t>
+          <t>"Others" Module Evidence 3/3 - Client's Sector</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">

</xml_diff>